<commit_message>
feat(repeat): round 4 = C2 H2 H5 I4 BIN5 aqueous; F3 and F4 stay as they are
The user's call: F3 and F4 fail the replicate screen but their means sit on block F's
trend, so they keep the two-point interval instead of a repeat. C2 joins: its aqueous
terpenes (1218 ppm) read above its own water-solvent edge (1018). 10 vials.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/repeat4_entry.xlsx
+++ b/out/repeat4_entry.xlsx
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P20"/>
+  <dimension ref="A1:P18"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -822,12 +822,12 @@
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>BIN5</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>BIN5-B1</t>
+          <t>C2-B1</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
@@ -874,12 +874,12 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>BIN5</t>
+          <t>C2</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>BIN5-B2</t>
+          <t>C2-B2</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -926,12 +926,12 @@
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>BIN5</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>F3-B1</t>
+          <t>BIN5-B1</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
@@ -978,12 +978,12 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>F3</t>
+          <t>BIN5</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>F3-B2</t>
+          <t>BIN5-B2</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
@@ -1030,17 +1030,17 @@
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>H2</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>F4-B1</t>
+          <t>H2-T1</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Inferior</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
@@ -1082,17 +1082,17 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>F4</t>
+          <t>H2</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>F4-B2</t>
+          <t>H2-T2</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Inferior</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -1134,17 +1134,17 @@
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>H2</t>
+          <t>H5</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>H2-T1</t>
+          <t>H5-B1</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
@@ -1186,17 +1186,17 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>H2</t>
+          <t>H5</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>H2-T2</t>
+          <t>H5-B2</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -1238,17 +1238,17 @@
     <row r="17">
       <c r="A17" s="11" t="inlineStr">
         <is>
-          <t>H5</t>
+          <t>I4</t>
         </is>
       </c>
       <c r="B17" s="11" t="inlineStr">
         <is>
-          <t>H5-B1</t>
+          <t>I4-T1</t>
         </is>
       </c>
       <c r="C17" s="11" t="inlineStr">
         <is>
-          <t>Inferior</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="D17" s="11" t="inlineStr">
@@ -1290,17 +1290,17 @@
     <row r="18">
       <c r="A18" s="3" t="inlineStr">
         <is>
-          <t>H5</t>
+          <t>I4</t>
         </is>
       </c>
       <c r="B18" s="3" t="inlineStr">
         <is>
-          <t>H5-B2</t>
+          <t>I4-T2</t>
         </is>
       </c>
       <c r="C18" s="3" t="inlineStr">
         <is>
-          <t>Inferior</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="D18" s="3" t="inlineStr">
@@ -1339,114 +1339,10 @@
       </c>
       <c r="P18" s="18" t="n"/>
     </row>
-    <row r="19">
-      <c r="A19" s="11" t="inlineStr">
-        <is>
-          <t>I4</t>
-        </is>
-      </c>
-      <c r="B19" s="11" t="inlineStr">
-        <is>
-          <t>I4-T1</t>
-        </is>
-      </c>
-      <c r="C19" s="11" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D19" s="11" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E19" s="12" t="n"/>
-      <c r="F19" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G19" s="12" t="n"/>
-      <c r="H19" s="11">
-        <f>1000-F19</f>
-        <v/>
-      </c>
-      <c r="I19" s="12" t="n"/>
-      <c r="J19" s="14">
-        <f>IF(AND(ISNUMBER(E19),ISNUMBER(G19)),G19-E19,"")</f>
-        <v/>
-      </c>
-      <c r="K19" s="14">
-        <f>IF(AND(ISNUMBER(G19),ISNUMBER(I19)),I19-G19,"")</f>
-        <v/>
-      </c>
-      <c r="L19" s="15">
-        <f>IF(AND(ISNUMBER(J19),ISNUMBER(K19)),IF(J19&gt;0,(J19+K19)/J19,""),"")</f>
-        <v/>
-      </c>
-      <c r="M19" s="16" t="n"/>
-      <c r="N19" s="16" t="n"/>
-      <c r="O19" s="11" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P19" s="13" t="n"/>
-    </row>
-    <row r="20">
-      <c r="A20" s="3" t="inlineStr">
-        <is>
-          <t>I4</t>
-        </is>
-      </c>
-      <c r="B20" s="3" t="inlineStr">
-        <is>
-          <t>I4-T2</t>
-        </is>
-      </c>
-      <c r="C20" s="3" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D20" s="3" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E20" s="17" t="n"/>
-      <c r="F20" s="18" t="n">
-        <v>300</v>
-      </c>
-      <c r="G20" s="17" t="n"/>
-      <c r="H20" s="3">
-        <f>1000-F20</f>
-        <v/>
-      </c>
-      <c r="I20" s="17" t="n"/>
-      <c r="J20" s="19">
-        <f>IF(AND(ISNUMBER(E20),ISNUMBER(G20)),G20-E20,"")</f>
-        <v/>
-      </c>
-      <c r="K20" s="19">
-        <f>IF(AND(ISNUMBER(G20),ISNUMBER(I20)),I20-G20,"")</f>
-        <v/>
-      </c>
-      <c r="L20" s="20">
-        <f>IF(AND(ISNUMBER(J20),ISNUMBER(K20)),IF(J20&gt;0,(J20+K20)/J20,""),"")</f>
-        <v/>
-      </c>
-      <c r="M20" s="5" t="n"/>
-      <c r="N20" s="5" t="n"/>
-      <c r="O20" s="3" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P20" s="18" t="n"/>
-    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <dataValidations count="1">
-    <dataValidation sqref="E9:G9 E10:G10 E11:G11 E12:G12 E13:G13 E14:G14 E15:G15 E16:G16 E17:G17 E18:G18 E19:G19 E20:G20 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18 I19 I20" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
+    <dataValidation sqref="E9:G9 E10:G10 E11:G11 E12:G12 E13:G13 E14:G14 E15:G15 E16:G16 E17:G17 E18:G18 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>

</xml_diff>

<commit_message>
feat(repeat): round 4 = H2 H5 I4 BIN5 aqueous; C2 stays
The user's call: C2's gap to its own edge (1218 +- 143 vs 1018 +- 93 ppm) is 1.17x their
combined U -- within experimental reach, not worth a tube. 8 vials.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
</commit_message>
<xml_diff>
--- a/out/repeat4_entry.xlsx
+++ b/out/repeat4_entry.xlsx
@@ -492,7 +492,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr fitToPage="1"/>
   </sheetPr>
-  <dimension ref="A1:P18"/>
+  <dimension ref="A1:P16"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="7" customWidth="1" min="1" max="1"/>
@@ -822,12 +822,12 @@
     <row r="9">
       <c r="A9" s="11" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>BIN5</t>
         </is>
       </c>
       <c r="B9" s="11" t="inlineStr">
         <is>
-          <t>C2-B1</t>
+          <t>BIN5-B1</t>
         </is>
       </c>
       <c r="C9" s="11" t="inlineStr">
@@ -874,12 +874,12 @@
     <row r="10">
       <c r="A10" s="3" t="inlineStr">
         <is>
-          <t>C2</t>
+          <t>BIN5</t>
         </is>
       </c>
       <c r="B10" s="3" t="inlineStr">
         <is>
-          <t>C2-B2</t>
+          <t>BIN5-B2</t>
         </is>
       </c>
       <c r="C10" s="3" t="inlineStr">
@@ -926,17 +926,17 @@
     <row r="11">
       <c r="A11" s="11" t="inlineStr">
         <is>
-          <t>BIN5</t>
+          <t>H2</t>
         </is>
       </c>
       <c r="B11" s="11" t="inlineStr">
         <is>
-          <t>BIN5-B1</t>
+          <t>H2-T1</t>
         </is>
       </c>
       <c r="C11" s="11" t="inlineStr">
         <is>
-          <t>Inferior</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="D11" s="11" t="inlineStr">
@@ -978,17 +978,17 @@
     <row r="12">
       <c r="A12" s="3" t="inlineStr">
         <is>
-          <t>BIN5</t>
+          <t>H2</t>
         </is>
       </c>
       <c r="B12" s="3" t="inlineStr">
         <is>
-          <t>BIN5-B2</t>
+          <t>H2-T2</t>
         </is>
       </c>
       <c r="C12" s="3" t="inlineStr">
         <is>
-          <t>Inferior</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="D12" s="3" t="inlineStr">
@@ -1030,17 +1030,17 @@
     <row r="13">
       <c r="A13" s="11" t="inlineStr">
         <is>
-          <t>H2</t>
+          <t>H5</t>
         </is>
       </c>
       <c r="B13" s="11" t="inlineStr">
         <is>
-          <t>H2-T1</t>
+          <t>H5-B1</t>
         </is>
       </c>
       <c r="C13" s="11" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D13" s="11" t="inlineStr">
@@ -1082,17 +1082,17 @@
     <row r="14">
       <c r="A14" s="3" t="inlineStr">
         <is>
-          <t>H2</t>
+          <t>H5</t>
         </is>
       </c>
       <c r="B14" s="3" t="inlineStr">
         <is>
-          <t>H2-T2</t>
+          <t>H5-B2</t>
         </is>
       </c>
       <c r="C14" s="3" t="inlineStr">
         <is>
-          <t>Superior</t>
+          <t>Inferior</t>
         </is>
       </c>
       <c r="D14" s="3" t="inlineStr">
@@ -1134,17 +1134,17 @@
     <row r="15">
       <c r="A15" s="11" t="inlineStr">
         <is>
-          <t>H5</t>
+          <t>I4</t>
         </is>
       </c>
       <c r="B15" s="11" t="inlineStr">
         <is>
-          <t>H5-B1</t>
+          <t>I4-T1</t>
         </is>
       </c>
       <c r="C15" s="11" t="inlineStr">
         <is>
-          <t>Inferior</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="D15" s="11" t="inlineStr">
@@ -1186,17 +1186,17 @@
     <row r="16">
       <c r="A16" s="3" t="inlineStr">
         <is>
-          <t>H5</t>
+          <t>I4</t>
         </is>
       </c>
       <c r="B16" s="3" t="inlineStr">
         <is>
-          <t>H5-B2</t>
+          <t>I4-T2</t>
         </is>
       </c>
       <c r="C16" s="3" t="inlineStr">
         <is>
-          <t>Inferior</t>
+          <t>Superior</t>
         </is>
       </c>
       <c r="D16" s="3" t="inlineStr">
@@ -1235,114 +1235,10 @@
       </c>
       <c r="P16" s="18" t="n"/>
     </row>
-    <row r="17">
-      <c r="A17" s="11" t="inlineStr">
-        <is>
-          <t>I4</t>
-        </is>
-      </c>
-      <c r="B17" s="11" t="inlineStr">
-        <is>
-          <t>I4-T1</t>
-        </is>
-      </c>
-      <c r="C17" s="11" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D17" s="11" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E17" s="12" t="n"/>
-      <c r="F17" s="13" t="n">
-        <v>300</v>
-      </c>
-      <c r="G17" s="12" t="n"/>
-      <c r="H17" s="11">
-        <f>1000-F17</f>
-        <v/>
-      </c>
-      <c r="I17" s="12" t="n"/>
-      <c r="J17" s="14">
-        <f>IF(AND(ISNUMBER(E17),ISNUMBER(G17)),G17-E17,"")</f>
-        <v/>
-      </c>
-      <c r="K17" s="14">
-        <f>IF(AND(ISNUMBER(G17),ISNUMBER(I17)),I17-G17,"")</f>
-        <v/>
-      </c>
-      <c r="L17" s="15">
-        <f>IF(AND(ISNUMBER(J17),ISNUMBER(K17)),IF(J17&gt;0,(J17+K17)/J17,""),"")</f>
-        <v/>
-      </c>
-      <c r="M17" s="16" t="n"/>
-      <c r="N17" s="16" t="n"/>
-      <c r="O17" s="11" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P17" s="13" t="n"/>
-    </row>
-    <row r="18">
-      <c r="A18" s="3" t="inlineStr">
-        <is>
-          <t>I4</t>
-        </is>
-      </c>
-      <c r="B18" s="3" t="inlineStr">
-        <is>
-          <t>I4-T2</t>
-        </is>
-      </c>
-      <c r="C18" s="3" t="inlineStr">
-        <is>
-          <t>Superior</t>
-        </is>
-      </c>
-      <c r="D18" s="3" t="inlineStr">
-        <is>
-          <t>aqueous</t>
-        </is>
-      </c>
-      <c r="E18" s="17" t="n"/>
-      <c r="F18" s="18" t="n">
-        <v>300</v>
-      </c>
-      <c r="G18" s="17" t="n"/>
-      <c r="H18" s="3">
-        <f>1000-F18</f>
-        <v/>
-      </c>
-      <c r="I18" s="17" t="n"/>
-      <c r="J18" s="19">
-        <f>IF(AND(ISNUMBER(E18),ISNUMBER(G18)),G18-E18,"")</f>
-        <v/>
-      </c>
-      <c r="K18" s="19">
-        <f>IF(AND(ISNUMBER(G18),ISNUMBER(I18)),I18-G18,"")</f>
-        <v/>
-      </c>
-      <c r="L18" s="20">
-        <f>IF(AND(ISNUMBER(J18),ISNUMBER(K18)),IF(J18&gt;0,(J18+K18)/J18,""),"")</f>
-        <v/>
-      </c>
-      <c r="M18" s="5" t="n"/>
-      <c r="N18" s="5" t="n"/>
-      <c r="O18" s="3" t="inlineStr">
-        <is>
-          <t>n/a: by difference</t>
-        </is>
-      </c>
-      <c r="P18" s="18" t="n"/>
-    </row>
   </sheetData>
   <sheetProtection selectLockedCells="0" selectUnlockedCells="0" sheet="1" objects="0" insertRows="1" insertHyperlinks="1" autoFilter="1" scenarios="0" formatColumns="1" deleteColumns="1" insertColumns="1" pivotTables="1" deleteRows="1" formatCells="1" formatRows="1" sort="1"/>
   <dataValidations count="1">
-    <dataValidation sqref="E9:G9 E10:G10 E11:G11 E12:G12 E13:G13 E14:G14 E15:G15 E16:G16 E17:G17 E18:G18 I9 I10 I11 I12 I13 I14 I15 I16 I17 I18" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
+    <dataValidation sqref="E9:G9 E10:G10 E11:G11 E12:G12 E13:G13 E14:G14 E15:G15 E16:G16 I9 I10 I11 I12 I13 I14 I15 I16" showDropDown="0" showInputMessage="0" showErrorMessage="1" allowBlank="0" error="A number between 0 and 100" type="decimal">
       <formula1>0</formula1>
       <formula2>100</formula2>
     </dataValidation>

</xml_diff>